<commit_message>
feat: auto-generacion de expedientes de personal al detectar nuevas personas en asistencia, checklist documental RH y blindaje on_click ignore
</commit_message>
<xml_diff>
--- a/personal.xlsx
+++ b/personal.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
   <si>
     <t>id_empleado</t>
   </si>
@@ -64,6 +64,18 @@
     <t>1145</t>
   </si>
   <si>
+    <t>1626</t>
+  </si>
+  <si>
+    <t>1636</t>
+  </si>
+  <si>
+    <t>1624</t>
+  </si>
+  <si>
+    <t>1625</t>
+  </si>
+  <si>
     <t>BRYAN ALEJANDRO FLORES MANCINAS</t>
   </si>
   <si>
@@ -101,6 +113,18 @@
   </si>
   <si>
     <t>ARMANDO WOO VAZQUEZ</t>
+  </si>
+  <si>
+    <t>CARREON LOPEZ  CRUZ</t>
+  </si>
+  <si>
+    <t>GARCIA LOERA  DAVID FERNANDO</t>
+  </si>
+  <si>
+    <t>MORENO RIOS  MAXIMILIANO</t>
+  </si>
+  <si>
+    <t>VAZQUEZ PADILLA  NATALY CRISTAL</t>
   </si>
   <si>
     <t>✂️ Corte Laser</t>
@@ -453,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -472,10 +496,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -483,10 +507,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -494,10 +518,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -505,10 +529,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -516,10 +540,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -527,10 +551,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -538,10 +562,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -549,10 +573,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -560,10 +584,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -571,10 +595,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -582,10 +606,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -593,10 +617,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -604,10 +628,54 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
         <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>